<commit_message>
Part list updated. word doc also updated with new ICs and comparison of XMC and AMIC.
</commit_message>
<xml_diff>
--- a/Documents/Dev-Files/Parts List/Parts List - Revised.xlsx
+++ b/Documents/Dev-Files/Parts List/Parts List - Revised.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\ChrisitanRaun-AnnanasMotor\Documents\Dev-Files\Parts List\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAA1B38C-5A5C-4C78-8063-926CA0F5E16F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6952EE58-20C5-4346-9F2A-E198BB672450}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{623B4204-36C6-4A79-936E-19F9F488D703}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="56">
   <si>
     <t>S.No</t>
   </si>
@@ -75,9 +75,6 @@
     <t>Encoder</t>
   </si>
   <si>
-    <t>AEAT-8800-Q24</t>
-  </si>
-  <si>
     <t>Rotary Magentic Encoder</t>
   </si>
   <si>
@@ -108,24 +105,12 @@
     <t>Header</t>
   </si>
   <si>
-    <t>M55-7012042R</t>
-  </si>
-  <si>
     <t>Debugging Header</t>
   </si>
   <si>
     <t>MagJack</t>
   </si>
   <si>
-    <t>Mouser</t>
-  </si>
-  <si>
-    <t>ARM Microcontrollers - MCU XMC4000</t>
-  </si>
-  <si>
-    <t>XMC4700F144K1536AAXQMA1</t>
-  </si>
-  <si>
     <t>HR915310A</t>
   </si>
   <si>
@@ -153,28 +138,61 @@
     <t>CHRISTIAN RAUN COMPONENTS LIST - Revised</t>
   </si>
   <si>
-    <t>LAN8700C-AEZG-TR</t>
-  </si>
-  <si>
-    <t>Ethernet tranceiver</t>
-  </si>
-  <si>
-    <t>Newark</t>
-  </si>
-  <si>
-    <t>MII/RMII 10/100 ETHERNET TRANSCEIVER 36 VQFN 6X6X1.0MM T/R ROHS COMPLIANT: YES</t>
-  </si>
-  <si>
     <t>Ethernet Connectors/Modular Connectors (RJ45)</t>
   </si>
   <si>
-    <t>IC BUS SWITCH 8 X 1:1 20VQFN</t>
-  </si>
-  <si>
-    <t>SN74CB3Q3245RGYR</t>
-  </si>
-  <si>
-    <t>Level Shifter</t>
+    <t>DC input jack</t>
+  </si>
+  <si>
+    <t>TLE5012BE5000FUMA1</t>
+  </si>
+  <si>
+    <t>DigiKey</t>
+  </si>
+  <si>
+    <t>LAN9255-I/ZMX019</t>
+  </si>
+  <si>
+    <t>IC ETHERCAT SLAVE CONTROLLER</t>
+  </si>
+  <si>
+    <t>SBH11-PBPC-D10-ST-BK</t>
+  </si>
+  <si>
+    <t>for 25 pieces. Price will decrease till $13 when ordered around 200 pieces.</t>
+  </si>
+  <si>
+    <t>ADC-028-1-T/R-PA10T</t>
+  </si>
+  <si>
+    <t>Power Barrel Connector Jack 2.00mm ID (0.079"), 5.50mm OD (0.217") Surface Mount, Right Angle</t>
+  </si>
+  <si>
+    <t>Screw terminals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Connector for a 4 wire stepper </t>
+  </si>
+  <si>
+    <t>Drive Mosfets</t>
+  </si>
+  <si>
+    <t>C3E-25.000-8-1015-X-M</t>
+  </si>
+  <si>
+    <t>CRYSTAL 25.0000MHZ 8PF SMD</t>
+  </si>
+  <si>
+    <t>Crystal</t>
+  </si>
+  <si>
+    <t>FDMC86106LZ</t>
+  </si>
+  <si>
+    <t>MOSFET N-CH 100V 3.3A POWER33</t>
+  </si>
+  <si>
+    <t>1-24 pieces</t>
   </si>
 </sst>
 </file>
@@ -184,7 +202,7 @@
   <numFmts count="1">
     <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -204,6 +222,12 @@
       <b/>
       <sz val="12"/>
       <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -347,63 +371,69 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -412,22 +442,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="12">
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
@@ -568,26 +582,42 @@
       </border>
     </dxf>
     <dxf>
-      <border>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
       </border>
     </dxf>
     <dxf>
-      <border diagonalUp="0" diagonalDown="0">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
         <right style="thin">
           <color indexed="64"/>
         </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <top/>
+        <bottom/>
       </border>
     </dxf>
   </dxfs>
@@ -604,15 +634,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{29E9361C-78C2-48C7-891A-B03AA0352AB1}" name="Table2" displayName="Table2" ref="A2:G18" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0" headerRowBorderDxfId="10" tableBorderDxfId="11" totalsRowBorderDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{29E9361C-78C2-48C7-891A-B03AA0352AB1}" name="Table2" displayName="Table2" ref="A2:G17" totalsRowShown="0" headerRowDxfId="11" dataDxfId="9" headerRowBorderDxfId="10" tableBorderDxfId="8" totalsRowBorderDxfId="7">
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{074CA092-EBD3-4E18-B22A-8F972F914B28}" name="S.No" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{18CB7E39-4265-430B-8777-0EE8A4B58655}" name="Component Name" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{45862D11-CD61-46FC-8326-308275CC6DB8}" name="Manufacturer Part Number" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{F992FF51-435A-4C58-AD4C-0699037533E8}" name="Description" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{96C0499C-A0FB-4857-859B-545A4547ABD9}" name="Reference URL" dataDxfId="4" dataCellStyle="Hyperlink"/>
-    <tableColumn id="6" xr3:uid="{F1CAF6DF-B8DC-4E9D-A60A-FD987F5B78D0}" name="Unit Cost" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{8B895613-6226-4609-92A1-19D9B147B311}" name="Remarks from Client" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{074CA092-EBD3-4E18-B22A-8F972F914B28}" name="S.No" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{18CB7E39-4265-430B-8777-0EE8A4B58655}" name="Component Name" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{45862D11-CD61-46FC-8326-308275CC6DB8}" name="Manufacturer Part Number" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{F992FF51-435A-4C58-AD4C-0699037533E8}" name="Description" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{96C0499C-A0FB-4857-859B-545A4547ABD9}" name="Reference URL" dataDxfId="2" dataCellStyle="Hyperlink"/>
+    <tableColumn id="6" xr3:uid="{F1CAF6DF-B8DC-4E9D-A60A-FD987F5B78D0}" name="Unit Cost" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{8B895613-6226-4609-92A1-19D9B147B311}" name="Remarks from Client" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -915,7 +945,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CB0C397-22AD-463F-8CBD-1AF936A9EBA0}">
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.5703125" customWidth="1"/>
@@ -928,326 +958,345 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" s="9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="10">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" s="3">
+        <v>6.63</v>
+      </c>
+      <c r="G3" s="11"/>
+    </row>
+    <row r="4" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A4" s="10">
+        <v>2</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" s="9" t="s">
+      <c r="D4" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F4" s="3">
+        <v>16.18</v>
+      </c>
+      <c r="G4" s="21" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="10">
         <v>3</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="B5" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F5" s="3">
+        <v>0.21</v>
+      </c>
+      <c r="G5" s="11"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="10">
         <v>4</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="B6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" s="3">
+        <v>0.65</v>
+      </c>
+      <c r="G6" s="11"/>
+    </row>
+    <row r="7" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="10">
         <v>5</v>
       </c>
-      <c r="G2" s="10" t="s">
+      <c r="B7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" s="3">
+        <v>2.46</v>
+      </c>
+      <c r="G7" s="11"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="10">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="11">
-        <v>1</v>
-      </c>
-      <c r="B3" s="2" t="s">
+      <c r="B8" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="3">
+        <v>0.2</v>
+      </c>
+      <c r="G8" s="11"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="10">
         <v>7</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="B9" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F9" s="3">
+        <v>0.43</v>
+      </c>
+      <c r="G9" s="11" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="10">
         <v>8</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="B10" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F10" s="3">
+        <v>0.45</v>
+      </c>
+      <c r="G10" s="11"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="10">
         <v>9</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="B11" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="4">
-        <v>6.63</v>
-      </c>
-      <c r="G3" s="12"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="11">
-        <v>2</v>
-      </c>
-      <c r="B4" s="2" t="s">
+      <c r="F11" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="G11" s="11"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="10">
+        <v>10</v>
+      </c>
+      <c r="B12" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F12" s="3">
+        <v>18.95</v>
+      </c>
+      <c r="G12" s="13"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="10">
         <v>11</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="F4" s="4">
-        <v>16.11</v>
-      </c>
-      <c r="G4" s="12"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="11">
+      <c r="B13" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F13" s="3">
+        <v>3.26</v>
+      </c>
+      <c r="G13" s="13"/>
+    </row>
+    <row r="14" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A14" s="10">
+        <v>12</v>
+      </c>
+      <c r="B14" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D14" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F14" s="6">
         <v>3</v>
       </c>
-      <c r="B5" s="16" t="s">
-        <v>36</v>
-      </c>
-      <c r="C5" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="D5" s="2" t="s">
+      <c r="G14" s="11"/>
+    </row>
+    <row r="15" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A15" s="10">
+        <v>13</v>
+      </c>
+      <c r="B15" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="E5" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="F5" s="4">
-        <v>0.21</v>
-      </c>
-      <c r="G5" s="12"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="11">
-        <v>4</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="2" t="s">
+      <c r="C15" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D15" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F15" s="3">
+        <v>0.8</v>
+      </c>
+      <c r="G15" s="11"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="10">
         <v>14</v>
       </c>
-      <c r="E6" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F6" s="4">
-        <v>0.65</v>
-      </c>
-      <c r="G6" s="12"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="11">
-        <v>5</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F7" s="4">
-        <v>9.36</v>
-      </c>
-      <c r="G7" s="12"/>
-    </row>
-    <row r="8" spans="1:7" ht="45" x14ac:dyDescent="0.25">
-      <c r="A8" s="11">
-        <v>6</v>
-      </c>
-      <c r="B8" s="18" t="s">
-        <v>43</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="D8" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="F8" s="7">
-        <v>1.82</v>
-      </c>
-      <c r="G8" s="12"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="11">
-        <v>7</v>
-      </c>
-      <c r="B9" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="C9" s="2" t="s">
+      <c r="B16" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="C16" s="1">
+        <v>1985218</v>
+      </c>
+      <c r="D16" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F9" s="4">
-        <v>0.88</v>
-      </c>
-      <c r="G9" s="12"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="11">
-        <v>8</v>
-      </c>
-      <c r="B10" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F10" s="4">
-        <v>0.45</v>
-      </c>
-      <c r="G10" s="12"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="11">
-        <v>9</v>
-      </c>
-      <c r="B11" s="16" t="s">
-        <v>26</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F11" s="4">
-        <v>1.34</v>
-      </c>
-      <c r="G11" s="12"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="11">
-        <v>10</v>
-      </c>
-      <c r="B12" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="F12" s="4">
-        <v>18.95</v>
-      </c>
-      <c r="G12" s="14"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="11">
-        <v>11</v>
-      </c>
-      <c r="B13" s="16" t="s">
-        <v>39</v>
-      </c>
-      <c r="C13" s="2" t="s">
+      <c r="E16" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D13" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F13" s="4">
-        <v>3.26</v>
-      </c>
-      <c r="G13" s="14"/>
-    </row>
-    <row r="14" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A14" s="11">
-        <v>12</v>
-      </c>
-      <c r="B14" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D14" s="19" t="s">
-        <v>46</v>
-      </c>
-      <c r="E14" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="F14" s="7">
-        <v>3</v>
-      </c>
-      <c r="G14" s="12"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="11"/>
-      <c r="B15" s="16"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="12"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="11"/>
-      <c r="B16" s="16"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="4"/>
-      <c r="G16" s="12"/>
+      <c r="F16" s="3">
+        <v>0.6</v>
+      </c>
+      <c r="G16" s="11"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="11"/>
-      <c r="B17" s="16"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="4"/>
-      <c r="G17" s="12"/>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="13"/>
-      <c r="B18" s="18"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="7"/>
-      <c r="G18" s="14"/>
+      <c r="A17" s="12"/>
+      <c r="B17" s="17"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1256,21 +1305,23 @@
   <hyperlinks>
     <hyperlink ref="E3" r:id="rId1" xr:uid="{26C41CE9-6DD4-417E-B327-9FEAF34153CA}"/>
     <hyperlink ref="E6" r:id="rId2" xr:uid="{4A8D8176-DFDF-4BE5-BF45-322C3D4261B7}"/>
-    <hyperlink ref="E7" r:id="rId3" xr:uid="{C32D6C63-BF95-4A72-AB73-55F6E42AD1F4}"/>
-    <hyperlink ref="E12" r:id="rId4" xr:uid="{06A9B98D-F6A0-451E-AE25-7582C35573FF}"/>
-    <hyperlink ref="E13" r:id="rId5" xr:uid="{05EAD26A-0BB8-4F3E-9D94-1A56DC8B5E06}"/>
-    <hyperlink ref="E11" r:id="rId6" xr:uid="{9FB9BE64-1577-475B-9811-D2A2A41C49BD}"/>
-    <hyperlink ref="E4" r:id="rId7" xr:uid="{E31C7531-1F66-4B6E-B4FE-763ED2A60F5E}"/>
-    <hyperlink ref="E14" r:id="rId8" xr:uid="{779ECD78-33EE-49DA-A32E-80F97346C34B}"/>
-    <hyperlink ref="E5" r:id="rId9" xr:uid="{965C0271-F5D8-439C-A055-4223ED6B5930}"/>
-    <hyperlink ref="E8" r:id="rId10" xr:uid="{B5EBF6B2-7A27-4B86-8232-C59C0348C9CD}"/>
-    <hyperlink ref="E10" r:id="rId11" xr:uid="{B32AEC71-2B64-4732-A393-F40A4AD5BD48}"/>
-    <hyperlink ref="E9" r:id="rId12" xr:uid="{C98B57A6-6A31-4966-819A-11BE1CE701CF}"/>
+    <hyperlink ref="E12" r:id="rId3" xr:uid="{06A9B98D-F6A0-451E-AE25-7582C35573FF}"/>
+    <hyperlink ref="E13" r:id="rId4" xr:uid="{05EAD26A-0BB8-4F3E-9D94-1A56DC8B5E06}"/>
+    <hyperlink ref="E4" r:id="rId5" xr:uid="{E31C7531-1F66-4B6E-B4FE-763ED2A60F5E}"/>
+    <hyperlink ref="E14" r:id="rId6" xr:uid="{779ECD78-33EE-49DA-A32E-80F97346C34B}"/>
+    <hyperlink ref="E5" r:id="rId7" xr:uid="{965C0271-F5D8-439C-A055-4223ED6B5930}"/>
+    <hyperlink ref="E10" r:id="rId8" xr:uid="{B32AEC71-2B64-4732-A393-F40A4AD5BD48}"/>
+    <hyperlink ref="E7" r:id="rId9" xr:uid="{C32D6C63-BF95-4A72-AB73-55F6E42AD1F4}"/>
+    <hyperlink ref="E11" r:id="rId10" xr:uid="{9FB9BE64-1577-475B-9811-D2A2A41C49BD}"/>
+    <hyperlink ref="E15" r:id="rId11" xr:uid="{18D7F878-86F5-417E-B342-D1A319A6B4A9}"/>
+    <hyperlink ref="E16" r:id="rId12" xr:uid="{00AA1C19-436A-4F64-AA4E-B82B03414973}"/>
+    <hyperlink ref="E8" r:id="rId13" xr:uid="{9293B878-7405-4DA0-BDE8-47C20655BEB3}"/>
+    <hyperlink ref="E9" r:id="rId14" xr:uid="{AB3A5CA8-FAA3-4E8C-AD4A-596D6E227D3A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId13"/>
+  <pageSetup orientation="portrait" r:id="rId15"/>
   <tableParts count="1">
-    <tablePart r:id="rId14"/>
+    <tablePart r:id="rId16"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>